<commit_message>
Lots of LS 0 models
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nihar/Desktop/Research/Similarity-Aware Label-Smoothing/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FE1F555-1B01-3442-9D1B-E57DA1EC2B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1383C9CB-8FD2-FA4B-9C37-22FE5645FA7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="68800" yWindow="20980" windowWidth="27040" windowHeight="16880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="27040" windowHeight="16860" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ResNET18" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="20">
   <si>
     <t>CIFAR-100</t>
   </si>
@@ -68,13 +68,29 @@
   </si>
   <si>
     <t>k = 10</t>
+  </si>
+  <si>
+    <t>epsilon = 0.01</t>
+  </si>
+  <si>
+    <t>epsilon = 0.005</t>
+  </si>
+  <si>
+    <t>epsilon = 0.2</t>
+  </si>
+  <si>
+    <t>epsilon = 0.02</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="170" formatCode="0.0000"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -89,16 +105,24 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="13"/>
-      <color rgb="FF000000"/>
-      <name val="Arial Unicode MS"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -125,10 +149,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -137,14 +162,8 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -152,8 +171,20 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -457,12 +488,12 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:M44"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="6.1640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.1640625" style="2" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7" style="2" bestFit="1" customWidth="1"/>
@@ -474,18 +505,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E1" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="J1" s="8" t="s">
+      <c r="E1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="J1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="K1" s="8"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="8"/>
+      <c r="K1" s="6"/>
+      <c r="L1" s="6"/>
+      <c r="M1" s="6"/>
     </row>
     <row r="2" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
@@ -517,23 +548,23 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
       <c r="C4" s="3">
         <v>0</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="8">
         <v>4.7500000000000001E-2</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="8">
         <v>0.878</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="8">
         <v>0.78390000000000004</v>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="8">
         <v>0.94420000000000004</v>
       </c>
     </row>
@@ -541,67 +572,122 @@
       <c r="C5" s="3">
         <v>14</v>
       </c>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
     </row>
     <row r="6" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C6" s="3">
         <v>2026</v>
       </c>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
     </row>
     <row r="7" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C7" s="3">
         <v>4212</v>
       </c>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
     </row>
     <row r="8" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C8" s="3">
         <v>50000</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+    </row>
+    <row r="9" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C9" s="3"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+    </row>
     <row r="10" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C10" s="3">
         <v>0</v>
       </c>
-      <c r="E10" s="2">
-        <v>8.9729465544223702E-2</v>
-      </c>
-      <c r="F10" s="2">
-        <v>0.95665431022643999</v>
-      </c>
-      <c r="G10" s="2">
-        <v>0.79779999999999995</v>
-      </c>
-      <c r="H10" s="2">
-        <v>0.94530000000000003</v>
-      </c>
+      <c r="E10" s="9">
+        <v>4.1314508765935898E-2</v>
+      </c>
+      <c r="F10" s="9">
+        <v>0.89415574073791504</v>
+      </c>
+      <c r="G10" s="9">
+        <v>0.78459999999999996</v>
+      </c>
+      <c r="H10" s="9">
+        <v>0.94399999999999995</v>
+      </c>
+      <c r="K10" s="3"/>
+      <c r="M10" s="9"/>
     </row>
     <row r="11" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" s="3">
-        <v>14</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="7"/>
+      <c r="K11" s="3"/>
+      <c r="M11" s="7"/>
     </row>
     <row r="12" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C12" s="3">
-        <v>2026</v>
-      </c>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
     </row>
     <row r="13" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
       <c r="C13" s="3">
-        <v>4212</v>
+        <v>0</v>
+      </c>
+      <c r="E13" s="9">
+        <v>4.4672753661870901E-2</v>
+      </c>
+      <c r="F13" s="9">
+        <v>0.893712878227233</v>
+      </c>
+      <c r="G13" s="9">
+        <v>0.79010000000000002</v>
+      </c>
+      <c r="H13" s="9">
+        <v>0.94330000000000003</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C14" s="3">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
+    </row>
+    <row r="15" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C15" s="3"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
+      <c r="H15" s="7"/>
+    </row>
     <row r="16" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>10</v>
@@ -609,67 +695,118 @@
       <c r="C16" s="3">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
+      <c r="H16" s="7"/>
+    </row>
+    <row r="17" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+      <c r="H17" s="7"/>
+    </row>
+    <row r="18" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C18" s="3"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="7"/>
+    </row>
+    <row r="19" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>8</v>
+      </c>
+      <c r="C19" s="3">
+        <v>0</v>
+      </c>
+      <c r="E19" s="9">
+        <v>8.9729465544223702E-2</v>
+      </c>
+      <c r="F19" s="9">
+        <v>0.95665431022643999</v>
+      </c>
+      <c r="G19" s="9">
+        <v>0.79779999999999995</v>
+      </c>
+      <c r="H19" s="9">
+        <v>0.94530000000000003</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C20" s="3"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+    </row>
+    <row r="21" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C21" s="3"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+    </row>
+    <row r="22" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="3">
+        <v>0</v>
+      </c>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+    </row>
+    <row r="23" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
         <v>11</v>
       </c>
-      <c r="C17" s="3">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C18" s="3">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C19" s="3">
-        <v>4212</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C20" s="3">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="22" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>12</v>
-      </c>
-      <c r="C22" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" s="3">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>13</v>
-      </c>
-      <c r="C24" s="3">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C23" s="3"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+    </row>
+    <row r="24" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C24" s="3"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+    </row>
+    <row r="25" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>8</v>
+      </c>
       <c r="C25" s="3">
-        <v>4212</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C26" s="3">
-        <v>50000</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="28" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+    </row>
+    <row r="26" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="3"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+    </row>
+    <row r="27" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="28" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>12</v>
       </c>
@@ -677,15 +814,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C29" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>13</v>
       </c>
@@ -693,12 +830,12 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="31" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C31" s="3">
         <v>4212</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:8" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C32" s="3">
         <v>50000</v>
       </c>
@@ -714,7 +851,7 @@
     </row>
     <row r="35" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C35" s="3">
         <v>14</v>
@@ -722,7 +859,7 @@
     </row>
     <row r="36" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C36" s="3">
         <v>2026</v>
@@ -740,50 +877,85 @@
     </row>
     <row r="39" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="40" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="5" t="s">
+      <c r="A40" t="s">
         <v>12</v>
       </c>
-      <c r="B40" s="5"/>
-      <c r="C40" s="6">
-        <v>0</v>
-      </c>
-      <c r="D40" s="5"/>
+      <c r="C40" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="41" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="5" t="s">
+      <c r="A41" t="s">
         <v>9</v>
       </c>
-      <c r="B41" s="5"/>
-      <c r="C41" s="6">
+      <c r="C41" s="3">
         <v>14</v>
       </c>
-      <c r="D41" s="5"/>
     </row>
     <row r="42" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="5" t="s">
+      <c r="A42" t="s">
+        <v>14</v>
+      </c>
+      <c r="C42" s="3">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C43" s="3">
+        <v>4212</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C44" s="3">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B46" s="10"/>
+      <c r="C46" s="11">
+        <v>0</v>
+      </c>
+      <c r="D46" s="4"/>
+    </row>
+    <row r="47" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B47" s="10"/>
+      <c r="C47" s="11">
+        <v>14</v>
+      </c>
+      <c r="D47" s="4"/>
+    </row>
+    <row r="48" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B42" s="5"/>
-      <c r="C42" s="6">
+      <c r="B48" s="10"/>
+      <c r="C48" s="11">
         <v>2026</v>
       </c>
-      <c r="D42" s="5"/>
-    </row>
-    <row r="43" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="5"/>
-      <c r="B43" s="5"/>
-      <c r="C43" s="6">
+      <c r="D48" s="4"/>
+    </row>
+    <row r="49" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="10"/>
+      <c r="B49" s="10"/>
+      <c r="C49" s="11">
         <v>4212</v>
       </c>
-      <c r="D43" s="5"/>
-    </row>
-    <row r="44" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5"/>
-      <c r="C44" s="6">
+      <c r="D49" s="4"/>
+    </row>
+    <row r="50" spans="1:4" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="10"/>
+      <c r="B50" s="10"/>
+      <c r="C50" s="11">
         <v>50000</v>
       </c>
-      <c r="D44" s="5"/>
+      <c r="D50" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>